<commit_message>
Actualización de Inventario de hallazgos 2.0
</commit_message>
<xml_diff>
--- a/InventarioDeHallazgos.xlsx
+++ b/InventarioDeHallazgos.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\quice\Documents\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tomax\OneDrive\Documentos\Universidad\6to Semestre\Arquitectura de software\Examen#1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{92FEF36B-E539-4134-A4BA-9E75F56E5FCF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F9CD525E-0029-4264-BD84-BA845757F765}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{35B2FC4D-D3EF-46AB-9279-816ECCC0806F}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="58">
   <si>
     <t>Inventario De Hallazgos</t>
   </si>
@@ -99,9 +99,6 @@
   </si>
   <si>
     <t>H-10</t>
-  </si>
-  <si>
-    <t>H-11</t>
   </si>
   <si>
     <t>OCP</t>
@@ -133,9 +130,6 @@
     <t>LSP</t>
   </si>
   <si>
-    <t>Media</t>
-  </si>
-  <si>
     <t>.\BibFarmacia\Servicios\ServicioProducto.cs
 Linea: 12</t>
   </si>
@@ -143,18 +137,12 @@
     <t>DIP</t>
   </si>
   <si>
-    <t xml:space="preserve">Alta </t>
-  </si>
-  <si>
     <t>Se mezcla lógica de presentación con lógica de negocio dentro de la misma clase.</t>
   </si>
   <si>
     <t>La clase se esta encargando de responsabilidad de otra capa (Presentacion). Esto reduce la claridad del código, incrementa el acoplamiento y dificulta el mantenimiento, las pruebas y la reutilización de la lógica de negocio.</t>
   </si>
   <si>
-    <t>Alta</t>
-  </si>
-  <si>
     <t>Los valores de StockMínimo, FechaVencimiento, TipoRelleno y MaterialEnvase están codificados directamente (hardcodeados) en los métodos de la fábrica.</t>
   </si>
   <si>
@@ -186,6 +174,60 @@
   </si>
   <si>
     <t>La validación termina desplazándose hacia los servicios o la lógica de aplicación, sobrecargando dichas capas y permitiendo que existan objetos en estados inválidos. Las entidades deberían proteger sus propias invariantes y garantizar su consistencia.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+.\BibFarmacia\Servicios\ServicioDescuento.cs
+ Linea: 15 
+</t>
+  </si>
+  <si>
+    <t>El metodo CalcularDescuento de la entinedad ServicioDescuento esta utilziando un porcentaje quemado para calcular el descuento</t>
+  </si>
+  <si>
+    <t>Cuando se quiera cambiar o agregar mas tipos de descuentos a la logica de negocio, habria que entrar a modificar el codigo de la clase y cambiar el procentaje dentor del metodo, lo que le quitaria flexibilidad y escalabilidad a nuevas modificaciones frente a la agregación de descuentos adicionales.</t>
+  </si>
+  <si>
+    <t>Alta/Propia</t>
+  </si>
+  <si>
+    <t>Alta/Asistida</t>
+  </si>
+  <si>
+    <t>Media/Asistida</t>
+  </si>
+  <si>
+    <t>Media/Propia</t>
+  </si>
+  <si>
+    <t>Baja/Asistida</t>
+  </si>
+  <si>
+    <t>Esta quemando la entidad de la cual se esta obteninedo el metodo para poder leer y logear los usuarios.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+.\BibFarmacia\Servicios\ServicioUsuario.cs
+ Linea: 31
+</t>
+  </si>
+  <si>
+    <t>Es costoso porque no permite que se pueda adaptar el codigo a un tipo de autenticación diferente, debido a que no recibe como parametro la clase que define que metodo de autenticación se usará. Esto crea alta complejidad a la hora de una migración de base de datos o donde se obtengan los usuarios</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+.\BibFarmacia\Enums\TipoRelleno.cs
+Linea: 7-14 
+</t>
+  </si>
+  <si>
+    <t>Se esta utilizando un enum para definir el tipo de relleno lo que limita el tipo de comportamiento que tiene cada uno de los tipos para rellenar el envase</t>
+  </si>
+  <si>
+    <t>El impacto que tiene para el negocio es que retrasa la implemetnación de nuevos tipos de relleno ya que hay que reestructurar la lista de los tipos existentes y para le metodo de como se rellena este tipo se tendria que entrar a modificar el codigo lo que implicaría posibles daños en estructuras que ya funcionan, lo que le resta modularidad al programa.</t>
+  </si>
+  <si>
+    <t>Alta/ Propia</t>
   </si>
 </sst>
 </file>
@@ -273,7 +315,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -296,6 +338,9 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -676,7 +721,7 @@
         <v>7</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C3" s="3"/>
       <c r="D3" s="3"/>
@@ -692,19 +737,19 @@
         <v>7</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="D4" s="7" t="s">
         <v>11</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="F4" s="6" t="s">
-        <v>35</v>
+        <v>46</v>
       </c>
     </row>
     <row r="5" spans="1:6" ht="72" x14ac:dyDescent="0.3">
@@ -712,19 +757,19 @@
         <v>10</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="D5" s="7" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>37</v>
+        <v>33</v>
       </c>
       <c r="F5" s="6" t="s">
-        <v>35</v>
+        <v>46</v>
       </c>
     </row>
     <row r="6" spans="1:6" ht="86.4" x14ac:dyDescent="0.3">
@@ -732,19 +777,19 @@
         <v>12</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="D6" s="7" t="s">
         <v>11</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="F6" s="6" t="s">
-        <v>35</v>
+        <v>46</v>
       </c>
     </row>
     <row r="7" spans="1:6" ht="86.4" x14ac:dyDescent="0.3">
@@ -752,19 +797,19 @@
         <v>13</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="D7" s="7" t="s">
         <v>11</v>
       </c>
       <c r="E7" s="4" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="F7" s="6" t="s">
-        <v>35</v>
+        <v>46</v>
       </c>
     </row>
     <row r="8" spans="1:6" ht="100.8" x14ac:dyDescent="0.3">
@@ -772,19 +817,19 @@
         <v>14</v>
       </c>
       <c r="B8" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="C8" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="D8" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="C8" s="4" t="s">
-        <v>40</v>
-      </c>
-      <c r="D8" s="7" t="s">
-        <v>28</v>
-      </c>
       <c r="E8" s="4" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="F8" s="6" t="s">
-        <v>29</v>
+        <v>48</v>
       </c>
     </row>
     <row r="9" spans="1:6" ht="72" x14ac:dyDescent="0.3">
@@ -792,19 +837,19 @@
         <v>15</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="D9" s="7" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="E9" s="4" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="F9" s="6" t="s">
-        <v>32</v>
+        <v>47</v>
       </c>
     </row>
     <row r="10" spans="1:6" ht="86.4" x14ac:dyDescent="0.3">
@@ -812,60 +857,80 @@
         <v>16</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="D10" s="6" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="E10" s="4" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="F10" s="6" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A11" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="B11" s="4"/>
-      <c r="C11" s="4"/>
-      <c r="D11" s="5"/>
-      <c r="E11" s="4"/>
-      <c r="F11" s="4"/>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="B11" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="C11" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="D11" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="E11" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="F11" s="6" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A12" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="B12" s="4"/>
-      <c r="C12" s="4"/>
-      <c r="D12" s="5"/>
-      <c r="E12" s="4"/>
-      <c r="F12" s="4"/>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="B12" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="C12" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="D12" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="E12" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="F12" s="6" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" ht="115.2" x14ac:dyDescent="0.3">
       <c r="A13" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="B13" s="4"/>
-      <c r="C13" s="4"/>
-      <c r="D13" s="5"/>
-      <c r="E13" s="4"/>
-      <c r="F13" s="4"/>
-    </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A14" s="5" t="s">
+      <c r="B13" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="C13" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="D13" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="B14" s="4"/>
-      <c r="C14" s="4"/>
-      <c r="D14" s="5"/>
-      <c r="E14" s="4"/>
-      <c r="F14" s="4"/>
+      <c r="E13" s="9" t="s">
+        <v>56</v>
+      </c>
+      <c r="F13" s="6" t="s">
+        <v>57</v>
+      </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A15" s="1"/>

</xml_diff>

<commit_message>
Actualización del inventario de hallazgos 3.0
</commit_message>
<xml_diff>
--- a/InventarioDeHallazgos.xlsx
+++ b/InventarioDeHallazgos.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tomax\OneDrive\Documentos\Universidad\6to Semestre\Arquitectura de software\Examen#1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F9CD525E-0029-4264-BD84-BA845757F765}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B98EF046-58F3-4524-B464-A8BCB43C5523}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{35B2FC4D-D3EF-46AB-9279-816ECCC0806F}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="58">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="63">
   <si>
     <t>Inventario De Hallazgos</t>
   </si>
@@ -227,7 +227,27 @@
     <t>El impacto que tiene para el negocio es que retrasa la implemetnación de nuevos tipos de relleno ya que hay que reestructurar la lista de los tipos existentes y para le metodo de como se rellena este tipo se tendria que entrar a modificar el codigo lo que implicaría posibles daños en estructuras que ya funcionan, lo que le resta modularidad al programa.</t>
   </si>
   <si>
-    <t>Alta/ Propia</t>
+    <t>H-11</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+.\BibFarmacia\Interfaces\IDescuento.cs
+Linea: 7-13
+.\BibFarmacia\Interfaces\IServicioNotificacion
+Linea: 7-13
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DIP </t>
+  </si>
+  <si>
+    <t>Rechazada/Asistida</t>
+  </si>
+  <si>
+    <t>La IA esta proponiendo que este fragemento de código, en este caso las interfaces, esta correcto porque se aplica el DIP pero en realidad esta afirmación no es correcta</t>
+  </si>
+  <si>
+    <t>El equipo decide refutar y rechazar esta idea de la IA debido a que en realidad estas interfaces solamente estan simulando que aplican DIP, porque unicamente se crean y se implementan cada una en un servicio de notificaciones y de descuento pero en ningun punto desacoplan clases entre sí, por lo que simplemente son fragmento de código innecesario en cuanto al cumplimiento del principio.</t>
   </si>
 </sst>
 </file>
@@ -315,7 +335,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -339,8 +359,14 @@
     <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -912,7 +938,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="13" spans="1:6" ht="115.2" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:6" ht="139.19999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="5" t="s">
         <v>19</v>
       </c>
@@ -925,11 +951,31 @@
       <c r="D13" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="E13" s="9" t="s">
+      <c r="E13" s="4" t="s">
         <v>56</v>
       </c>
       <c r="F13" s="6" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" ht="124.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A14" s="11" t="s">
         <v>57</v>
+      </c>
+      <c r="B14" s="10" t="s">
+        <v>58</v>
+      </c>
+      <c r="C14" s="10" t="s">
+        <v>61</v>
+      </c>
+      <c r="D14" s="9" t="s">
+        <v>59</v>
+      </c>
+      <c r="E14" s="10" t="s">
+        <v>62</v>
+      </c>
+      <c r="F14" s="11" t="s">
+        <v>60</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
Arreglo de inventario de hallazgos
</commit_message>
<xml_diff>
--- a/InventarioDeHallazgos.xlsx
+++ b/InventarioDeHallazgos.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tomax\OneDrive\Documentos\Universidad\6to Semestre\Arquitectura de software\Examen#1\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/145dae6a10ca7481/Escritorio/Universidad/Semestre 6/Arquitectura Software/Examen 1/SolucionFarmacia/SolucionFarmacia/docs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B98EF046-58F3-4524-B464-A8BCB43C5523}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="3" documentId="13_ncr:1_{B98EF046-58F3-4524-B464-A8BCB43C5523}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{748F638A-A87A-425E-9B9E-975DF639958F}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{35B2FC4D-D3EF-46AB-9279-816ECCC0806F}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{35B2FC4D-D3EF-46AB-9279-816ECCC0806F}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="63">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="65">
   <si>
     <t>Inventario De Hallazgos</t>
   </si>
@@ -63,12 +63,6 @@
   </si>
   <si>
     <t>H-01</t>
-  </si>
-  <si>
-    <t>Traducido a costo, riesgo o tiempo de cambio</t>
-  </si>
-  <si>
-    <t>Alta / Media / Baja — Propio o Asistido</t>
   </si>
   <si>
     <t>H-02</t>
@@ -117,10 +111,11 @@
   </si>
   <si>
     <t>.\BibFarmacia\Servicios\ServicioProducto.cs
-Linea: 25, 42, 75</t>
-  </si>
-  <si>
-    <t>.\BibFarmacia\Clases\</t>
+Linea: 27, 42, 75</t>
+  </si>
+  <si>
+    <t>.\BibFarmacia\Clases\Producto.cs
+Linea: 10-14</t>
   </si>
   <si>
     <t>.\BibFarmacia\Clases\Medicamento.cs
@@ -131,7 +126,7 @@
   </si>
   <si>
     <t>.\BibFarmacia\Servicios\ServicioProducto.cs
-Linea: 12</t>
+Linea: 14, 16-17, 93-107</t>
   </si>
   <si>
     <t>DIP</t>
@@ -200,15 +195,12 @@
     <t>Media/Propia</t>
   </si>
   <si>
-    <t>Baja/Asistida</t>
-  </si>
-  <si>
     <t>Esta quemando la entidad de la cual se esta obteninedo el metodo para poder leer y logear los usuarios.</t>
   </si>
   <si>
     <t xml:space="preserve">
 .\BibFarmacia\Servicios\ServicioUsuario.cs
- Linea: 31
+ Linea: 29-33
 </t>
   </si>
   <si>
@@ -233,7 +225,7 @@
     <t xml:space="preserve">
 .\BibFarmacia\Interfaces\IDescuento.cs
 Linea: 7-13
-.\BibFarmacia\Interfaces\IServicioNotificacion
+.\BibFarmacia\Interfaces\IServicioNotificacion.cs
 Linea: 7-13
 </t>
   </si>
@@ -248,6 +240,22 @@
   </si>
   <si>
     <t>El equipo decide refutar y rechazar esta idea de la IA debido a que en realidad estas interfaces solamente estan simulando que aplican DIP, porque unicamente se crean y se implementan cada una en un servicio de notificaciones y de descuento pero en ningun punto desacoplan clases entre sí, por lo que simplemente son fragmento de código innecesario en cuanto al cumplimiento del principio.</t>
+  </si>
+  <si>
+    <t>H-12</t>
+  </si>
+  <si>
+    <t>.\BibFarmacia\Servicios\ServicioProducto.cs
+Linea: 93-107</t>
+  </si>
+  <si>
+    <t>CargarDesdeArchivo siempre construye un MedicamentoCapsula con TipoRelleno.Gel fijo, sin importar el contenido real del archivo (no hay despacho por tipo de producto), y ademas hardcodea la direccion y el telefono del laboratorio ('Medellin', '4444444') en lugar de leerlos del archivo.</t>
+  </si>
+  <si>
+    <t>OCP / SRP</t>
+  </si>
+  <si>
+    <t>La carga de datos no puede crear ningun tipo de producto distinto a un medicamento en capsula, osea que cada nuevo tipo de producto obligaria a modificar este metodo. Ademas, los datos de laboratorio quedan incorrectos para todo lo cargado desde archivo, por lo que hay un riesgo de integridad de datos.</t>
   </si>
 </sst>
 </file>
@@ -335,14 +343,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -356,9 +361,6 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -367,6 +369,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -383,6 +388,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -702,27 +711,27 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AC02423B-4662-448E-B2F2-627D385E326A}">
-  <dimension ref="A1:F18"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:F17"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="2" max="2" width="43.109375" customWidth="1"/>
-    <col min="3" max="3" width="35.88671875" customWidth="1"/>
-    <col min="4" max="4" width="14.5546875" customWidth="1"/>
-    <col min="5" max="5" width="42.88671875" customWidth="1"/>
+    <col min="2" max="2" width="43.08984375" customWidth="1"/>
+    <col min="3" max="3" width="35.90625" customWidth="1"/>
+    <col min="4" max="4" width="14.54296875" customWidth="1"/>
+    <col min="5" max="5" width="42.90625" customWidth="1"/>
     <col min="6" max="6" width="18" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A1" s="8" t="s">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A1" s="10" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="8"/>
-      <c r="C1" s="8"/>
-      <c r="D1" s="8"/>
-      <c r="E1" s="8"/>
-      <c r="F1" s="8"/>
-    </row>
-    <row r="2" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="B1" s="10"/>
+      <c r="C1" s="10"/>
+      <c r="D1" s="10"/>
+      <c r="E1" s="10"/>
+      <c r="F1" s="10"/>
+    </row>
+    <row r="2" spans="1:6" ht="29" x14ac:dyDescent="0.35">
       <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
@@ -742,243 +751,247 @@
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A3" s="3" t="s">
+    <row r="3" spans="1:6" ht="72.5" x14ac:dyDescent="0.35">
+      <c r="A3" s="4" t="s">
         <v>7</v>
       </c>
       <c r="B3" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="D3" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="F3" s="5" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" ht="72.5" x14ac:dyDescent="0.35">
+      <c r="A4" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="D4" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="F4" s="5" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" ht="87" x14ac:dyDescent="0.35">
+      <c r="A5" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="B5" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="C3" s="3"/>
-      <c r="D3" s="3"/>
-      <c r="E3" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="F3" s="3" t="s">
+      <c r="C5" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="D5" s="6" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="4" spans="1:6" ht="72" x14ac:dyDescent="0.3">
-      <c r="A4" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="B4" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="C4" s="4" t="s">
-        <v>30</v>
-      </c>
-      <c r="D4" s="7" t="s">
+      <c r="E5" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="F5" s="5" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" ht="87" x14ac:dyDescent="0.35">
+      <c r="A6" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="E4" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="F4" s="6" t="s">
+      <c r="B6" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="D6" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="E6" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="F6" s="5" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" ht="101.5" x14ac:dyDescent="0.35">
+      <c r="A7" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="D7" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="E7" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="F7" s="5" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="5" spans="1:6" ht="72" x14ac:dyDescent="0.3">
-      <c r="A5" s="5" t="s">
-        <v>10</v>
-      </c>
-      <c r="B5" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="C5" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="D5" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="E5" s="4" t="s">
-        <v>33</v>
-      </c>
-      <c r="F5" s="6" t="s">
+    <row r="8" spans="1:6" ht="87" x14ac:dyDescent="0.35">
+      <c r="A8" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="D8" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="E8" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="F8" s="5" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" ht="87" x14ac:dyDescent="0.35">
+      <c r="A9" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="C9" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="D9" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="E9" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="F9" s="5" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="6" spans="1:6" ht="86.4" x14ac:dyDescent="0.3">
-      <c r="A6" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="B6" s="4" t="s">
-        <v>23</v>
-      </c>
-      <c r="C6" s="4" t="s">
-        <v>34</v>
-      </c>
-      <c r="D6" s="7" t="s">
-        <v>11</v>
-      </c>
-      <c r="E6" s="4" t="s">
-        <v>35</v>
-      </c>
-      <c r="F6" s="6" t="s">
+    <row r="10" spans="1:6" ht="101.5" x14ac:dyDescent="0.35">
+      <c r="A10" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="C10" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="D10" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="E10" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="F10" s="5" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="7" spans="1:6" ht="86.4" x14ac:dyDescent="0.3">
-      <c r="A7" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="B7" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="C7" s="4" t="s">
-        <v>34</v>
-      </c>
-      <c r="D7" s="7" t="s">
-        <v>11</v>
-      </c>
-      <c r="E7" s="4" t="s">
-        <v>35</v>
-      </c>
-      <c r="F7" s="6" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" ht="100.8" x14ac:dyDescent="0.3">
-      <c r="A8" s="5" t="s">
-        <v>14</v>
-      </c>
-      <c r="B8" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="C8" s="4" t="s">
-        <v>36</v>
-      </c>
-      <c r="D8" s="7" t="s">
+    <row r="11" spans="1:6" ht="101.5" x14ac:dyDescent="0.35">
+      <c r="A11" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="B11" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="C11" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="D11" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="E8" s="4" t="s">
-        <v>37</v>
-      </c>
-      <c r="F8" s="6" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6" ht="72" x14ac:dyDescent="0.3">
-      <c r="A9" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="B9" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="C9" s="4" t="s">
-        <v>38</v>
-      </c>
-      <c r="D9" s="7" t="s">
-        <v>29</v>
-      </c>
-      <c r="E9" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="F9" s="6" t="s">
+      <c r="E11" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="F11" s="5" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="10" spans="1:6" ht="86.4" x14ac:dyDescent="0.3">
-      <c r="A10" s="5" t="s">
-        <v>16</v>
-      </c>
-      <c r="B10" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="C10" s="4" t="s">
-        <v>40</v>
-      </c>
-      <c r="D10" s="6" t="s">
-        <v>41</v>
-      </c>
-      <c r="E10" s="4" t="s">
-        <v>42</v>
-      </c>
-      <c r="F10" s="6" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="11" spans="1:6" ht="100.8" x14ac:dyDescent="0.3">
-      <c r="A11" s="5" t="s">
+    <row r="12" spans="1:6" ht="139.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A12" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="B11" s="4" t="s">
-        <v>43</v>
-      </c>
-      <c r="C11" s="4" t="s">
+      <c r="B12" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="C12" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="D12" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="E12" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="F12" s="5" t="s">
         <v>44</v>
       </c>
-      <c r="D11" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="E11" s="4" t="s">
+    </row>
+    <row r="13" spans="1:6" ht="124.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A13" s="9" t="s">
+        <v>54</v>
+      </c>
+      <c r="B13" s="8" t="s">
+        <v>55</v>
+      </c>
+      <c r="C13" s="8" t="s">
+        <v>58</v>
+      </c>
+      <c r="D13" s="7" t="s">
+        <v>56</v>
+      </c>
+      <c r="E13" s="8" t="s">
+        <v>59</v>
+      </c>
+      <c r="F13" s="9" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" ht="116" x14ac:dyDescent="0.35">
+      <c r="A14" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="B14" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="C14" s="3" t="s">
+        <v>62</v>
+      </c>
+      <c r="D14" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="E14" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="F14" s="5" t="s">
         <v>45</v>
       </c>
-      <c r="F11" s="6" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="12" spans="1:6" ht="100.8" x14ac:dyDescent="0.3">
-      <c r="A12" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="B12" s="4" t="s">
-        <v>52</v>
-      </c>
-      <c r="C12" s="4" t="s">
-        <v>51</v>
-      </c>
-      <c r="D12" s="7" t="s">
-        <v>29</v>
-      </c>
-      <c r="E12" s="4" t="s">
-        <v>53</v>
-      </c>
-      <c r="F12" s="6" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="13" spans="1:6" ht="139.19999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="B13" s="4" t="s">
-        <v>54</v>
-      </c>
-      <c r="C13" s="4" t="s">
-        <v>55</v>
-      </c>
-      <c r="D13" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="E13" s="4" t="s">
-        <v>56</v>
-      </c>
-      <c r="F13" s="6" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="14" spans="1:6" ht="124.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="11" t="s">
-        <v>57</v>
-      </c>
-      <c r="B14" s="10" t="s">
-        <v>58</v>
-      </c>
-      <c r="C14" s="10" t="s">
-        <v>61</v>
-      </c>
-      <c r="D14" s="9" t="s">
-        <v>59</v>
-      </c>
-      <c r="E14" s="10" t="s">
-        <v>62</v>
-      </c>
-      <c r="F14" s="11" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A15" s="1"/>
       <c r="B15" s="1"/>
       <c r="C15" s="1"/>
@@ -986,7 +999,7 @@
       <c r="E15" s="1"/>
       <c r="F15" s="1"/>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A16" s="1"/>
       <c r="B16" s="1"/>
       <c r="C16" s="1"/>
@@ -994,21 +1007,13 @@
       <c r="E16" s="1"/>
       <c r="F16" s="1"/>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A17" s="1"/>
       <c r="B17" s="1"/>
       <c r="C17" s="1"/>
       <c r="D17" s="1"/>
       <c r="E17" s="1"/>
       <c r="F17" s="1"/>
-    </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A18" s="1"/>
-      <c r="B18" s="1"/>
-      <c r="C18" s="1"/>
-      <c r="D18" s="1"/>
-      <c r="E18" s="1"/>
-      <c r="F18" s="1"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>